<commit_message>
Changed footnotes i.e. numbering and new urban/rural classification
</commit_message>
<xml_diff>
--- a/reference-files/figures-template.xlsx
+++ b/reference-files/figures-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\irf\18-End-of-Life\Publication\Sissi\end-of-life-pub\reference-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64226FB3-9A08-4381-BDD4-F35BCB4FE637}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1832CA8-CC19-4516-905A-B8965E2E4F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" tabRatio="672" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="672" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="9" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="177">
   <si>
     <t>External causes of death excluded from analysis</t>
   </si>
@@ -552,9 +552,6 @@
     <t>The length of hospital stays in 2020/21 and 2021/22 are likely to have been impacted by measures in place at different stages of the COVID-19 pandemic. This may be an underlying reason for the larger increase in the percentage of time spent at home or in a community setting between 2019/20 and 2020/21.</t>
   </si>
   <si>
-    <t>https://www.gov.scot/publications/scottish-government-urban-rural-classification-2020/pages/0/</t>
-  </si>
-  <si>
     <t>45-54</t>
   </si>
   <si>
@@ -562,9 +559,6 @@
   </si>
   <si>
     <t>0-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. For more information on Urban / Rural classification see </t>
   </si>
   <si>
     <t>1. The NHS Board of Residence is the usual place of residence prior to death.</t>
@@ -586,6 +580,21 @@
   </si>
   <si>
     <t>1. Data are analysed by the 2020 ‘Scotland level’ Scottish Index of Multiple Deprivation (SIMD) population weighted quintiles. Each quintile consists of approximately 20% of the population living in Scotland, with deprivation quintile 1 indicating the population living in the most deprived areas.</t>
+  </si>
+  <si>
+    <t>https://www.gov.scot/publications/scottish-government-urban-rural-classification-2022</t>
+  </si>
+  <si>
+    <t>1. The 2022 Urban Rural classification has been used in this analysis.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> For more information on Urban / Rural classification see </t>
+  </si>
+  <si>
+    <t>1. The 2022 Urban Rural classification has been used in this analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For more information on Urban / Rural classification see </t>
   </si>
 </sst>
 </file>
@@ -3659,7 +3668,7 @@
     <row r="13" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="16" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -3815,7 +3824,7 @@
     <row r="18" spans="1:28" s="19" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" s="90" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C18" s="100" t="e">
         <f ca="1" xml:space="preserve"> calculation!B15</f>
@@ -4411,7 +4420,7 @@
         <v>80</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" spans="1:16" s="16" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
@@ -4542,7 +4551,7 @@
   <sheetPr codeName="Sheet10">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:M36"/>
+  <dimension ref="B1:M37"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="53" customWidth="1"/>
@@ -4597,7 +4606,7 @@
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
@@ -4612,11 +4621,16 @@
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B36" s="96" t="s">
-        <v>166</v>
-      </c>
-      <c r="G36" s="28" t="s">
-        <v>162</v>
+      <c r="B36" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="96" t="s">
+        <v>174</v>
+      </c>
+      <c r="G37" s="28" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -4626,7 +4640,7 @@
   <hyperlinks>
     <hyperlink ref="B31" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
     <hyperlink ref="B31:F31" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0900-000001000000}"/>
-    <hyperlink ref="G36" r:id="rId1" xr:uid="{00000000-0004-0000-0900-000002000000}"/>
+    <hyperlink ref="G37" r:id="rId1" xr:uid="{00000000-0004-0000-0900-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="90" orientation="landscape" r:id="rId2"/>
@@ -4639,7 +4653,7 @@
   <sheetPr codeName="Sheet11">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:S19"/>
+  <dimension ref="B1:S20"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="53" customWidth="1"/>
@@ -4787,7 +4801,7 @@
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -4817,10 +4831,15 @@
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="96" t="s">
-        <v>166</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>162</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="96" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" s="28" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -4830,7 +4849,7 @@
   <hyperlinks>
     <hyperlink ref="B14" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
     <hyperlink ref="B14:J14" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0A00-000001000000}"/>
-    <hyperlink ref="D19" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-000002000000}"/>
+    <hyperlink ref="D20" r:id="rId1" xr:uid="{00000000-0004-0000-0A00-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="92" orientation="landscape" r:id="rId2"/>
@@ -28935,7 +28954,7 @@
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
@@ -29268,7 +29287,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B21" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -29359,7 +29378,7 @@
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
@@ -29369,18 +29388,18 @@
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "1. " &amp; calculation!$B$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B39" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -29689,7 +29708,7 @@
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
@@ -29711,14 +29730,14 @@
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B26" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="J26" s="7"/>
       <c r="K26" s="7"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
@@ -29831,7 +29850,7 @@
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
@@ -29841,7 +29860,7 @@
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "1. " &amp; calculation!$B$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -29929,13 +29948,13 @@
         <v>153</v>
       </c>
       <c r="C7" s="80" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D7" s="80" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E7" s="80" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F7" s="80" t="s">
         <v>100</v>
@@ -30099,7 +30118,7 @@
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
@@ -30115,7 +30134,7 @@
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "1. " &amp; calculation!$B$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
         <v>#REF!</v>
       </c>
       <c r="J16" s="7"/>
@@ -30227,7 +30246,7 @@
     </row>
     <row r="3" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="91" t="e">
-        <f ca="1" xml:space="preserve"> "by Deprivation Category" &amp; calculation!$B$6 &amp; "; "  &amp; [0]!fy_max &amp; calculation!$B$5</f>
+        <f ca="1" xml:space="preserve"> "by Deprivation Category" &amp; calculation!$B$5 &amp; "; "  &amp; [0]!fy_max &amp; calculation!$B$4</f>
         <v>#REF!</v>
       </c>
     </row>
@@ -30255,7 +30274,7 @@
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -30273,13 +30292,13 @@
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "1. " &amp; calculation!$B$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="34" spans="2:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="108" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C34" s="108"/>
       <c r="D34" s="108"/>
@@ -30391,7 +30410,7 @@
     </row>
     <row r="3" spans="2:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="91" t="e">
-        <f ca="1" xml:space="preserve"> "by Deprivation Category" &amp; calculation!$B$6 &amp; "; "  &amp; [0]!fy_max &amp; calculation!$B$5</f>
+        <f ca="1" xml:space="preserve"> "by Deprivation Category" &amp; calculation!$B$5 &amp; "; "  &amp; [0]!fy_max &amp; calculation!$B$4</f>
         <v>#REF!</v>
       </c>
       <c r="C3" s="1"/>
@@ -30535,7 +30554,7 @@
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" s="96" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
@@ -30553,13 +30572,13 @@
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "1. " &amp; calculation!$B$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="108" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C18" s="108"/>
       <c r="D18" s="108"/>
@@ -30594,4 +30613,10 @@
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{b4199b9c-a89e-442f-9799-431511f14748}" enabled="1" method="Privileged" siteId="{10efe0bd-a030-4bca-809c-b5e6745e499a}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Added changes because of 2025 Annual Pub
</commit_message>
<xml_diff>
--- a/reference-files/figures-template.xlsx
+++ b/reference-files/figures-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stats\irf\18-End-of-Life\Publication\Sissi\end-of-life-pub\reference-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1832CA8-CC19-4516-905A-B8965E2E4F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B5A981-39A0-4BDE-9DDB-F39DD5A5DDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="672" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="672" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="9" r:id="rId1"/>
@@ -38,7 +38,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="11">'External Causes of Deaths'!$A$2:$E$49</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Figure 1'!$B$1:$L$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">OFFSET('Figure 1 Background Data'!$B$1:$H$1, 0, 0, calculation!$B$7+14, 9)</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Figure 2'!$B$1:$M$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Figure 2'!$B$1:$M$41</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Figure 2 Background Data'!$B$1:$J$27</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Figure 3'!$B$1:$M$32</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Figure 3 Background Data'!$B$1:$J$16</definedName>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="179">
   <si>
     <t>External causes of death excluded from analysis</t>
   </si>
@@ -274,9 +274,6 @@
   </si>
   <si>
     <t>Surgical and other medical procedures as the cause of abnormal reaction of the patient, or of later complication, without mention of misadventure at the time of the procedure</t>
-  </si>
-  <si>
-    <t>Source: International Statistical Classification of Diseases and Related Health Problems (10th Revision) 2007</t>
   </si>
   <si>
     <t>Quality Outcome Measure 10: Percentage of time in the last 6 months of life spent at home or in a community setting</t>
@@ -540,9 +537,6 @@
     <t>COVID-19 footnote</t>
   </si>
   <si>
-    <t>These statistics are derived from data collected on discharges from acute and community hospitals (SMR01), geriatric long stay facilities (SMR01 GLS) and pyschiatric hospitals (SMR04) in Scotland.</t>
-  </si>
-  <si>
     <t>Please note that people who died where a fall is coded on the death record are included within the cohort; W00-W19 Falls</t>
   </si>
   <si>
@@ -595,6 +589,18 @@
   </si>
   <si>
     <t xml:space="preserve">For more information on Urban / Rural classification see </t>
+  </si>
+  <si>
+    <t>These statistics are derived from data collected on discharges from acute and community hospitals (SMR01), geriatric long stay facilities (SMR01 GLS) and pyschiatric hospitals (SMR04) in Scotland. Figures for the last year are provisional.</t>
+  </si>
+  <si>
+    <t>Provisional note for latest f. year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See data completeness tables in Appendix 2 of report. </t>
+  </si>
+  <si>
+    <t>Source: International Statistical Classification of Diseases and Related Health Problems (11th Revision) 2024</t>
   </si>
 </sst>
 </file>
@@ -903,7 +909,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
@@ -1115,6 +1121,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="7" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="15">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2569,8 +2579,35 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="Arial"/>
             </a:rPr>
-            <a:t>= % of time at home or in a community 				               setting in last 6 months of life x 182.5</a:t>
+            <a:t>= (% of time at home or in a community 				                                                                    setting in last 6 months of life x 182.5) / 100</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr sz="1000"/>
+          </a:pPr>
+          <a:endParaRPr lang="en-GB" sz="1000" b="0" i="0" u="none" strike="noStrike" baseline="0">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Arial"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="Arial"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr algn="l" rtl="0">
@@ -3107,11 +3144,12 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AB78"/>
-  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="70" customWidth="1"/>
     <col min="2" max="2" width="3.44140625" style="70" customWidth="1"/>
-    <col min="3" max="256" width="9.109375" style="70"/>
+    <col min="3" max="13" width="11.5546875" style="70" customWidth="1"/>
+    <col min="14" max="256" width="9.109375" style="70"/>
     <col min="257" max="257" width="1.6640625" style="70" customWidth="1"/>
     <col min="258" max="258" width="3.44140625" style="70" customWidth="1"/>
     <col min="259" max="512" width="9.109375" style="70"/>
@@ -3323,7 +3361,7 @@
     <row r="2" spans="1:28" s="19" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="16"/>
       <c r="B2" s="14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="16"/>
@@ -3385,7 +3423,7 @@
     <row r="4" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="16"/>
       <c r="B4" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="16"/>
       <c r="D4" s="16"/>
@@ -3480,7 +3518,7 @@
     <row r="7" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="16"/>
       <c r="B7" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -3512,7 +3550,7 @@
     <row r="8" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -3544,7 +3582,7 @@
     <row r="9" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="16"/>
       <c r="B9" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -3576,7 +3614,7 @@
     <row r="10" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="16"/>
       <c r="B10" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -3668,7 +3706,7 @@
     <row r="13" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16"/>
       <c r="B13" s="16" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -3700,7 +3738,7 @@
     <row r="14" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="16"/>
       <c r="B14" s="19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
@@ -3762,7 +3800,7 @@
     <row r="16" spans="1:28" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="16"/>
       <c r="B16" s="20" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
@@ -3824,7 +3862,7 @@
     <row r="18" spans="1:28" s="19" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="16"/>
       <c r="B18" s="90" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C18" s="100" t="e">
         <f ca="1" xml:space="preserve"> calculation!B15</f>
@@ -3860,7 +3898,7 @@
       <c r="A19" s="16"/>
       <c r="B19" s="63"/>
       <c r="C19" s="102" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D19" s="102"/>
       <c r="E19" s="102"/>
@@ -3921,10 +3959,10 @@
     <row r="21" spans="1:28" s="19" customFormat="1" ht="28.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="16"/>
       <c r="B21" s="64" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C21" s="103" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D21" s="103"/>
       <c r="E21" s="103"/>
@@ -3984,10 +4022,10 @@
     </row>
     <row r="23" spans="1:28" s="16" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="64" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C23" s="97" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D23" s="97"/>
       <c r="E23" s="97"/>
@@ -4379,10 +4417,10 @@
     </row>
     <row r="46" spans="2:16" s="16" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="64" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C46" s="65" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D46" s="49"/>
       <c r="E46" s="49"/>
@@ -4417,16 +4455,16 @@
     </row>
     <row r="48" spans="2:16" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B48" s="88" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C48" s="16" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="49" spans="1:16" s="16" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B49" s="67"/>
       <c r="C49" s="68" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D49" s="5"/>
       <c r="E49" s="5"/>
@@ -4440,7 +4478,7 @@
     <row r="50" spans="1:16" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B50" s="26"/>
       <c r="C50" s="21" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D50" s="22"/>
       <c r="E50" s="23"/>
@@ -4457,10 +4495,10 @@
     </row>
     <row r="52" spans="1:16" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B52" s="89" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C52" s="16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:16" s="16" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
@@ -4470,10 +4508,10 @@
     <row r="54" spans="1:16" s="16" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="64"/>
       <c r="B54" s="90" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C54" s="98" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="D54" s="98"/>
       <c r="E54" s="98"/>
@@ -4492,6 +4530,9 @@
     <row r="55" spans="1:16" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="64"/>
       <c r="B55" s="64"/>
+      <c r="C55" s="2" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="56" spans="1:16" s="16" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="B56" s="63"/>
@@ -4538,11 +4579,12 @@
     <hyperlink ref="C19:P19" r:id="rId2" display="See Appendix 2 of the full report for more information." xr:uid="{DAB81432-778B-43DC-BFBA-4A4235F898E9}"/>
     <hyperlink ref="B6" location="'Figure 1'!A1" display="Figure 1: Percentage of time in the last six months of life spent at home or in a community setting (2010/11 - 2016/17)" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="B6:M6" location="'Figure 1'!A1" display="Figure 1: Percentage of time in the last six months of life spent at home or in a community setting (by age and gender)" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="C55" r:id="rId3" xr:uid="{062AD267-1B57-48DB-8776-38C20F6B03C1}"/>
   </hyperlinks>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="72" orientation="landscape" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="72" orientation="landscape" r:id="rId4"/>
   <headerFooter alignWithMargins="0"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -4577,7 +4619,7 @@
     </row>
     <row r="2" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
@@ -4606,12 +4648,12 @@
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B33" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B34" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.25">
@@ -4622,15 +4664,15 @@
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B36" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B37" s="96" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="G37" s="28" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -4690,7 +4732,7 @@
     </row>
     <row r="2" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -4715,7 +4757,7 @@
     </row>
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" s="44" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C6" s="35" t="e">
         <f ca="1">CONCATENATE([0]!fy_max, calculation!$B$4)</f>
@@ -4724,7 +4766,7 @@
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B7" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C7" s="45" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "urban rural 6", $B7), [0]!data_range, 5, FALSE)</f>
@@ -4733,7 +4775,7 @@
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B8" s="39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C8" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "urban rural 6", $B8), [0]!data_range, 5, FALSE)</f>
@@ -4742,7 +4784,7 @@
     </row>
     <row r="9" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B9" s="39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C9" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "urban rural 6", $B9), [0]!data_range, 5, FALSE)</f>
@@ -4751,7 +4793,7 @@
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" s="39" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C10" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "urban rural 6", $B10), [0]!data_range, 5, FALSE)</f>
@@ -4760,7 +4802,7 @@
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B11" s="39" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C11" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "urban rural 6", $B11), [0]!data_range, 5, FALSE)</f>
@@ -4769,7 +4811,7 @@
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B12" s="41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C12" s="47" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "urban rural 6", $B12), [0]!data_range, 5, FALSE)</f>
@@ -4801,7 +4843,7 @@
     </row>
     <row r="16" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B16" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -4813,7 +4855,7 @@
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
@@ -4831,15 +4873,15 @@
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="96" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="96" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D20" s="28" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -5650,7 +5692,7 @@
     <row r="44" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="25"/>
       <c r="B44" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="45" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -5659,13 +5701,13 @@
     <row r="46" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
       <c r="B46" s="13" t="s">
-        <v>70</v>
+        <v>178</v>
       </c>
     </row>
     <row r="47" spans="1:3" s="7" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="25"/>
       <c r="B47" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C47" s="2"/>
     </row>
@@ -6494,22 +6536,22 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
+        <v>110</v>
+      </c>
+      <c r="B1" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="C1" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="D1" s="29" t="s">
         <v>113</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="E1" s="29" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="F1" s="29" t="s">
         <v>115</v>
-      </c>
-      <c r="F1" s="29" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -28649,7 +28691,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1" s="30">
         <f>COUNTA(data!B:B)-1</f>
@@ -28658,7 +28700,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B2" s="30">
         <f>COUNTA(data!1:1)</f>
@@ -28667,33 +28709,33 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B4" s="48" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5" s="30" t="s">
         <v>129</v>
-      </c>
-      <c r="B5" s="30" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="29" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6" s="85" t="s">
         <v>144</v>
-      </c>
-      <c r="B6" s="85" t="s">
-        <v>145</v>
       </c>
       <c r="I6" s="29"/>
       <c r="K6" s="29"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B7" s="30">
         <v>10</v>
@@ -28804,15 +28846,15 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="B13" s="29" t="s">
         <v>136</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B14" s="30" t="e">
         <f ca="1">"Data for "&amp; $K$9 &amp;" are provisional. Please see Notes tab for more information."</f>
@@ -28821,7 +28863,7 @@
     </row>
     <row r="15" spans="1:11" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="50" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B15" s="111" t="e">
         <f ca="1">IF($B$13 = "provisional", "Hospital data and ", "") &amp; "National Records of Scotland deaths data " &amp; IF($B$13 = "provisional", "are", "is") &amp; " provisional for " &amp; $K$9 &amp;". " &amp; IF($B$13 = "provisional", "This publication will be updated in October 20" &amp; RIGHT($K$9,2) &amp; ". " &amp; $B$16, "")</f>
@@ -28837,10 +28879,10 @@
     </row>
     <row r="16" spans="1:11" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B16" s="112" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C16" s="111"/>
       <c r="D16" s="111"/>
@@ -28867,7 +28909,7 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="29" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B19" s="30" t="str">
         <f>"Figures in 2020/21 and 2021/22 are likely to have been affected by the impact of COVID-19 on hospital stays."</f>
@@ -28875,7 +28917,13 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="29"/>
+      <c r="A20" s="113" t="s">
+        <v>176</v>
+      </c>
+      <c r="B20" s="114" t="e">
+        <f ca="1">"Data for "&amp; $K$9 &amp;" are provisional. Please see Notes tab for more information. Where hospital completeness is lower, this may impact the amount of time spent at home or in the community."</f>
+        <v>#REF!</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="29"/>
@@ -28928,7 +28976,7 @@
     </row>
     <row r="2" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -28954,12 +29002,12 @@
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -29018,7 +29066,7 @@
     </row>
     <row r="2" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.6" x14ac:dyDescent="0.3">
@@ -29032,7 +29080,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C6" s="105" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D6" s="105"/>
       <c r="E6" s="24"/>
@@ -29040,13 +29088,13 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B7" s="75" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D7" s="35" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E7" s="24"/>
       <c r="F7" s="24"/>
@@ -29287,12 +29335,12 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B21" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -29326,7 +29374,7 @@
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:M40"/>
+  <dimension ref="B1:M41"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.6640625" style="53" customWidth="1"/>
@@ -29351,7 +29399,7 @@
     </row>
     <row r="2" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
@@ -29378,37 +29426,45 @@
     </row>
     <row r="36" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B36" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B37" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B38" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
+      <c r="B38" s="115" t="e">
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$20</f>
         <v>#REF!</v>
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="3" t="s">
-        <v>165</v>
+      <c r="B39" s="116" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B40" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:M1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B39" r:id="rId1" xr:uid="{6180DF36-5832-42B4-B47B-B1DED21040C1}"/>
+  </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="72" orientation="landscape" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" scale="72" orientation="landscape" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -29440,7 +29496,7 @@
     </row>
     <row r="2" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="2:11" ht="15.6" x14ac:dyDescent="0.3">
@@ -29454,7 +29510,7 @@
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="57" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C5" s="58" t="e">
         <f ca="1">CONCATENATE([0]!fy_max, calculation!$B$4)</f>
@@ -29469,7 +29525,7 @@
     </row>
     <row r="6" spans="2:11" ht="16.2" x14ac:dyDescent="0.25">
       <c r="B6" s="59" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C6" s="45" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B6), [0]!data_range, 5, FALSE)</f>
@@ -29484,7 +29540,7 @@
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="48" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C7" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B7), [0]!data_range, 5, FALSE)</f>
@@ -29499,7 +29555,7 @@
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="48" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C8" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B8), [0]!data_range, 5, FALSE)</f>
@@ -29514,7 +29570,7 @@
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="48" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C9" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B9), [0]!data_range, 5, FALSE)</f>
@@ -29529,7 +29585,7 @@
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="48" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C10" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B10), [0]!data_range, 5, FALSE)</f>
@@ -29545,7 +29601,7 @@
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="48" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C11" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B11), [0]!data_range, 5, FALSE)</f>
@@ -29561,7 +29617,7 @@
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="48" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C12" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B12), [0]!data_range, 5, FALSE)</f>
@@ -29577,7 +29633,7 @@
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B13), [0]!data_range, 5, FALSE)</f>
@@ -29593,7 +29649,7 @@
     </row>
     <row r="14" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B14" s="48" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C14" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B14), [0]!data_range, 5, FALSE)</f>
@@ -29609,7 +29665,7 @@
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C15" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B15), [0]!data_range, 5, FALSE)</f>
@@ -29625,7 +29681,7 @@
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" s="48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C16" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B16), [0]!data_range, 5, FALSE)</f>
@@ -29641,7 +29697,7 @@
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B17" s="48" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C17" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B17), [0]!data_range, 5, FALSE)</f>
@@ -29657,7 +29713,7 @@
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B18" s="48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C18" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B18), [0]!data_range, 5, FALSE)</f>
@@ -29673,7 +29729,7 @@
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B19" s="60" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" s="61" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "hb", $B19), [0]!data_range, 5, FALSE)</f>
@@ -29708,41 +29764,44 @@
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B23" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J23" s="7"/>
       <c r="K23" s="7"/>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J24" s="7"/>
       <c r="K24" s="7"/>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B25" s="3" t="e">
-        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$14</f>
+        <f ca="1" xml:space="preserve"> "p. " &amp; calculation!$B$20</f>
         <v>#REF!</v>
       </c>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="3" t="s">
-        <v>165</v>
+      <c r="B26" s="116" t="s">
+        <v>177</v>
       </c>
       <c r="J26" s="7"/>
       <c r="K26" s="7"/>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B27" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B28" s="3" t="s">
+        <v>167</v>
+      </c>
       <c r="J28" s="7"/>
       <c r="K28" s="7"/>
     </row>
@@ -29785,9 +29844,10 @@
   <hyperlinks>
     <hyperlink ref="B21" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
     <hyperlink ref="B21:E21" location="'External Causes of Deaths'!A1" display="External causes of death excluded from analysis" xr:uid="{00000000-0004-0000-0400-000001000000}"/>
+    <hyperlink ref="B26" r:id="rId1" xr:uid="{D513D6B8-1346-4D26-A9C2-BA4F33DD77C8}"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="90" verticalDpi="90" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="90" verticalDpi="90" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -29821,7 +29881,7 @@
     </row>
     <row r="2" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
@@ -29850,12 +29910,12 @@
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B30" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
@@ -29911,7 +29971,7 @@
     </row>
     <row r="2" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="2:19" ht="15.6" x14ac:dyDescent="0.3">
@@ -29931,7 +29991,7 @@
     <row r="6" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B6" s="48"/>
       <c r="C6" s="107" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D6" s="107"/>
       <c r="E6" s="107"/>
@@ -29945,31 +30005,31 @@
     </row>
     <row r="7" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B7" s="79" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C7" s="80" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D7" s="80" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E7" s="80" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F7" s="80" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" s="80" t="s">
         <v>100</v>
       </c>
-      <c r="G7" s="80" t="s">
+      <c r="H7" s="80" t="s">
         <v>101</v>
       </c>
-      <c r="H7" s="80" t="s">
+      <c r="I7" s="80" t="s">
         <v>102</v>
       </c>
-      <c r="I7" s="80" t="s">
+      <c r="J7" s="80" t="s">
         <v>103</v>
-      </c>
-      <c r="J7" s="80" t="s">
-        <v>104</v>
       </c>
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
@@ -29977,7 +30037,7 @@
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B8" s="48" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C8" s="93" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "age/sex", C$7, " ", $B8), [0]!data_range, 5, FALSE)</f>
@@ -30017,7 +30077,7 @@
     </row>
     <row r="9" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B9" s="48" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" s="93" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "age/sex", C$7, " ", $B9), [0]!data_range, 5, FALSE)</f>
@@ -30057,7 +30117,7 @@
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B10" s="81" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="94" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "age/sex", C$7, " ", $B10), [0]!data_range, 5, FALSE)</f>
@@ -30118,7 +30178,7 @@
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B14" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
@@ -30126,7 +30186,7 @@
     </row>
     <row r="15" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="J15" s="7"/>
       <c r="K15" s="7"/>
@@ -30241,7 +30301,7 @@
     </row>
     <row r="2" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="15.6" x14ac:dyDescent="0.3">
@@ -30274,7 +30334,7 @@
     </row>
     <row r="31" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B31" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
@@ -30283,7 +30343,7 @@
     </row>
     <row r="32" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B32" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
@@ -30298,7 +30358,7 @@
     </row>
     <row r="34" spans="2:13" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="108" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C34" s="108"/>
       <c r="D34" s="108"/>
@@ -30314,10 +30374,10 @@
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B35" s="96" t="s">
+        <v>106</v>
+      </c>
+      <c r="G35" s="28" t="s">
         <v>107</v>
-      </c>
-      <c r="G35" s="28" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.25">
@@ -30398,7 +30458,7 @@
     </row>
     <row r="2" spans="2:20" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="91" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -30431,7 +30491,7 @@
     </row>
     <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="42" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C6" s="43" t="e">
         <f ca="1">CONCATENATE([0]!fy_max, calculation!$B$4)</f>
@@ -30446,7 +30506,7 @@
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7" s="83" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C7" s="46" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "simd quintile", $B7), [0]!data_range, 5, FALSE)</f>
@@ -30506,7 +30566,7 @@
     </row>
     <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11" s="84" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C11" s="47" t="e">
         <f ca="1">VLOOKUP(CONCATENATE([0]!fy_max, "simd quintile", $B11), [0]!data_range, 5, FALSE)</f>
@@ -30554,7 +30614,7 @@
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" s="96" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C15" s="5"/>
       <c r="D15" s="5"/>
@@ -30563,7 +30623,7 @@
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C16" s="5"/>
       <c r="D16" s="5"/>
@@ -30578,7 +30638,7 @@
     </row>
     <row r="18" spans="2:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="108" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C18" s="108"/>
       <c r="D18" s="108"/>
@@ -30594,10 +30654,10 @@
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" s="96" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" s="28" t="s">
         <v>107</v>
-      </c>
-      <c r="E19" s="28" t="s">
-        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>